<commit_message>
feat(booking): implement tournament booking creation and management APIs
</commit_message>
<xml_diff>
--- a/Endpoint_desc.xlsx
+++ b/Endpoint_desc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sprort_Court_Managerment\PRN232-Project-Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B13C9ECB-E091-4A56-BDC1-06707ADC7288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C976B2C-ECA9-40F6-AB8D-BDEFB8388945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="81">
   <si>
     <t>STT</t>
   </si>
@@ -303,6 +303,66 @@
 {
   "message": "Quy định hệ thống: Khách hàng không được phép hủy sân. Vui lòng liên hệ hỗ trợ nếu bạn cần đổi sân hoặc khung giờ."
 }</t>
+  </si>
+  <si>
+    <t>Booking</t>
+  </si>
+  <si>
+    <t>/api/bookings/tournament</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>Tạo đơn đặt giải đấu (nhiều sân, nhiều khung giờ)</t>
+  </si>
+  <si>
+    <t>CreateTournamentRequest</t>
+  </si>
+  <si>
+    <t>TournamentDto</t>
+  </si>
+  <si>
+    <t>Tournament</t>
+  </si>
+  <si>
+    <t>/api/bookings/tournament/my</t>
+  </si>
+  <si>
+    <t>TournamentDto[]</t>
+  </si>
+  <si>
+    <t>/api/bookings/tournament/admin</t>
+  </si>
+  <si>
+    <t>Admin, Staff</t>
+  </si>
+  <si>
+    <t>Query: date, status</t>
+  </si>
+  <si>
+    <t>/api/bookings/tournament/{id}</t>
+  </si>
+  <si>
+    <t>Customer (own), Admin, Staff</t>
+  </si>
+  <si>
+    <t>TournamentDto (includes bookings, courts, slots, services)</t>
+  </si>
+  <si>
+    <t>/api/bookings/tournament/{id}/status</t>
+  </si>
+  <si>
+    <t>UpdateTournamentStatusRequest</t>
+  </si>
+  <si>
+    <t>/api/bookings/tournament/{id}/info</t>
+  </si>
+  <si>
+    <t>Customer (owner)</t>
+  </si>
+  <si>
+    <t>UpdateTournamentInfoRequest</t>
   </si>
 </sst>
 </file>
@@ -727,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1076,6 +1136,138 @@
         <v>60</v>
       </c>
     </row>
+    <row r="14" spans="1:8" ht="74.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="s">
+        <v>62</v>
+      </c>
+      <c r="E14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" t="s">
+        <v>64</v>
+      </c>
+      <c r="G14" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E15" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" t="s">
+        <v>74</v>
+      </c>
+      <c r="H17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" t="s">
+        <v>77</v>
+      </c>
+      <c r="H18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" t="s">
+        <v>80</v>
+      </c>
+      <c r="H19" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>